<commit_message>
recupere archivo pago y adema cambie la interfaz de pago a empleado
</commit_message>
<xml_diff>
--- a/Inventario.xlsx
+++ b/Inventario.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>FechaIngreso</t>
   </si>
@@ -30,21 +30,6 @@
   </si>
   <si>
     <t>ValorTotal</t>
-  </si>
-  <si>
-    <t>2024-10-31  Hora:  12:29</t>
-  </si>
-  <si>
-    <t>hols</t>
-  </si>
-  <si>
-    <t>2024-10-31</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>9.0</t>
   </si>
 </sst>
 </file>
@@ -89,7 +74,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -112,26 +97,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
elimine extraer en el tareas y reportes y borre unas imagenes
</commit_message>
<xml_diff>
--- a/Inventario.xlsx
+++ b/Inventario.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="47">
   <si>
     <t>FechaIngreso</t>
   </si>
@@ -144,6 +144,15 @@
   </si>
   <si>
     <t>10000</t>
+  </si>
+  <si>
+    <t>2024-11-13  Hora:  09:32</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>5000</t>
   </si>
 </sst>
 </file>
@@ -188,7 +197,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -391,6 +400,26 @@
         <v>21</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>